<commit_message>
Prepare MineralChain GitHub repository and AI models
</commit_message>
<xml_diff>
--- a/backend-minier/experiments/experimentation_results.xlsx
+++ b/backend-minier/experiments/experimentation_results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthese" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparaisons" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Synthese" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comparaisons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Meta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,10 +415,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -1310,6 +1310,686 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:10.699Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TC-04 Auto-validation d'un lot conforme DGMR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Partiellement conforme</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Validation DGMR on-chain observee avec statut AUTHENTIQUE</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:11.260Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TC-08 Mise a jour du certificat IPFS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Le hash IPFS du certificat a bien ete mis a jour</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:11.785Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TC-05 Detection d'un lot suspect</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KCC-2603-999</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>KCC</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>cobalt</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Le lot suspect a ete valide avec le statut SUSPECT</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:12.273Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TC-07 Controles d'acces onlyOwner</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Le contrat bloque bien validateByDGMR depuis un compte non owner</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:12.526Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TC-06 Prevention de double certification</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Le second mint du meme lot est correctement bloque</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:30.222Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TC-04 Auto-validation d'un lot conforme DGMR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Partiellement conforme</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Validation DGMR on-chain observee avec statut AUTHENTIQUE</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:31.280Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TC-08 Mise a jour du certificat IPFS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Le hash IPFS du certificat a bien ete mis a jour</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:32.284Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TC-05 Detection d'un lot suspect</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KCC-2603-999</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>KCC</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>cobalt</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Le lot suspect a ete valide avec le statut SUSPECT</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:33.283Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TC-07 Controles d'acces onlyOwner</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Le contrat bloque bien validateByDGMR depuis un compte non owner</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:34.104Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TC-06 Prevention de double certification</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nft-minier.truffle</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>truffle</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Le second mint du meme lot est correctement bloque</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1321,10 +2001,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -1767,6 +2447,346 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:10.699Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TC-04 Auto-validation d'un lot conforme DGMR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Partiellement conforme</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:11.260Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TC-08 Mise a jour du certificat IPFS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:11.785Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TC-05 Detection d'un lot suspect</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KCC-2603-999</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KCC</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:12.273Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TC-07 Controles d'acces onlyOwner</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:23:12.526Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TC-06 Prevention de double certification</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:30.222Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TC-04 Auto-validation d'un lot conforme DGMR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Partiellement conforme</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:31.280Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TC-08 Mise a jour du certificat IPFS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:32.284Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TC-05 Detection d'un lot suspect</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KCC-2603-999</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KCC</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:33.283Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TC-07 Controles d'acces onlyOwner</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:27:34.104Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TC-06 Prevention de double certification</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KAMOA-2603-142</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KAMOA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1806,7 +2826,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-24T09:54:49.414247</t>
+          <t>2026-05-22T13:27:34.712102</t>
         </is>
       </c>
     </row>
@@ -1817,7 +2837,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">

</xml_diff>